<commit_message>
fix: context dropdown rejected every value in hardware-calc.xlsx
Reported from the classroom: picking a context in C10 raised 'the value entered
must be an element of the specified list'.

A literal list validation ("2048,4096,...") is compared as TEXT, but the cell
holds a NUMBER -- and the thousands format rendered it as '8.192' on top of
that -- so no option ever matched. Numeric dropdowns must validate against a
range of numbers, so the context sizes now live in Referencia!H5:H11 and C10
points there; the cell format drops the thousands separator.

verifica-xlsx.py now cross-checks every list validation against its source
(literal or range) and fails when a numeric cell is validated against a literal
list, so this cannot come back.
</commit_message>
<xml_diff>
--- a/c1/hardware-calc.xlsx
+++ b/c1/hardware-calc.xlsx
@@ -263,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -295,16 +295,12 @@
     <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -342,8 +338,14 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -996,7 +998,7 @@
           <t>Usuaris simultanis</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="13" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -1004,7 +1006,7 @@
           <t>Hi cap?</t>
         </is>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="15">
         <f>IF($F$11&lt;0,"✘ No",IF($F$11&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
@@ -1029,7 +1031,7 @@
           <t>Amplada de banda (GB/s)</t>
         </is>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="16">
         <f>VLOOKUP($C$13,GPUs!$B$5:$H$14,3,FALSE)</f>
         <v/>
       </c>
@@ -1046,7 +1048,7 @@
           <t>t/s teòrics</t>
         </is>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <f>IF($F$7=0,0,VLOOKUP($C$13,GPUs!$B$5:$H$14,3,FALSE)/$F$7)</f>
         <v/>
       </c>
@@ -1058,11 +1060,11 @@
           <t>t/s esperats a la pràctica</t>
         </is>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="18">
         <f>$F$15*0.7</f>
         <v/>
       </c>
-      <c r="H16" s="20" t="n"/>
+      <c r="H16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="E17" s="2" t="inlineStr">
@@ -1079,21 +1081,21 @@
       </c>
     </row>
     <row r="19">
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="20" t="inlineStr">
         <is>
           <t>VRAM_pesos ≈ paràmetres (B) × bytes/paràmetre × 1,1</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="H20" s="21" t="inlineStr">
+      <c r="H20" s="20" t="inlineStr">
         <is>
           <t>tokens/s ≈ amplada de banda (GB/s) ÷ mida del model (GB)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>CIDET · IA en local · Classe 1</t>
         </is>
@@ -1136,7 +1138,7 @@
       <formula1>Referencia!$B$5:$B$9</formula1>
     </dataValidation>
     <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Context no vàlid" error="Tria una de les mides de context de la llista." type="list">
-      <formula1>"2048,4096,8192,16384,32768,65536,131072"</formula1>
+      <formula1>Referencia!$H$5:$H$11</formula1>
     </dataValidation>
     <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor no vàlid" error="Només 'No' o 'Q8'." type="list">
       <formula1>"No,Q8"</formula1>
@@ -1186,329 +1188,329 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>GPU</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>VRAM (GB)</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Amplada banda (GB/s)</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>Any</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Accelera FP8/FP4</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Preu orientatiu (€)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>RTX 3060</t>
         </is>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="24" t="n">
         <v>360</v>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Ampere</t>
         </is>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="24" t="n">
         <v>2021</v>
       </c>
-      <c r="G5" s="26" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H5" s="25" t="n">
+      <c r="H5" s="24" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="24" t="n">
         <v>672</v>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="E6" s="25" t="inlineStr">
         <is>
           <t>Blackwell</t>
         </is>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="24" t="n">
         <v>2025</v>
       </c>
-      <c r="G6" s="26" t="inlineStr">
+      <c r="G6" s="25" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="H6" s="24" t="n">
         <v>650</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>RTX 5060 Ti</t>
         </is>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="24" t="n">
         <v>448</v>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Blackwell</t>
         </is>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="24" t="n">
         <v>2025</v>
       </c>
-      <c r="G7" s="26" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H7" s="24" t="n">
         <v>480</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>RTX 4090</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="27" t="n">
         <v>1008</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>Ada Lovelace</t>
         </is>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="27" t="n">
         <v>2022</v>
       </c>
-      <c r="G8" s="29" t="inlineStr">
+      <c r="G8" s="28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="27" t="n">
         <v>1900</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="27" t="n">
         <v>1792</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
         <is>
           <t>Blackwell</t>
         </is>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="27" t="n">
         <v>2025</v>
       </c>
-      <c r="G9" s="29" t="inlineStr">
+      <c r="G9" s="28" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="H9" s="27" t="n">
         <v>2400</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>L4</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>Ada Lovelace</t>
         </is>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="27" t="n">
         <v>2023</v>
       </c>
-      <c r="G10" s="29" t="inlineStr">
+      <c r="G10" s="28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="27" t="n">
         <v>2600</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>A100 40GB</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="27" t="n">
         <v>1555</v>
       </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Ampere</t>
         </is>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="27" t="n">
         <v>2020</v>
       </c>
-      <c r="G11" s="29" t="inlineStr">
+      <c r="G11" s="28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H11" s="28" t="n">
+      <c r="H11" s="27" t="n">
         <v>9000</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>RTX 4060 Ti 16GB</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="27" t="n">
         <v>288</v>
       </c>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Ada Lovelace</t>
         </is>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="27" t="n">
         <v>2023</v>
       </c>
-      <c r="G12" s="29" t="inlineStr">
+      <c r="G12" s="28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="27" t="n">
         <v>480</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>RTX 3090</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="27" t="n">
         <v>936</v>
       </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="E13" s="28" t="inlineStr">
         <is>
           <t>Ampere</t>
         </is>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="27" t="n">
         <v>2020</v>
       </c>
-      <c r="G13" s="29" t="inlineStr">
+      <c r="G13" s="28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H13" s="28" t="n">
+      <c r="H13" s="27" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>RTX 5080</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="E14" s="29" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>Blackwell</t>
         </is>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="27" t="n">
         <v>2025</v>
       </c>
-      <c r="G14" s="29" t="inlineStr">
+      <c r="G14" s="28" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H14" s="28" t="n">
+      <c r="H14" s="27" t="n">
         <v>1200</v>
       </c>
     </row>
@@ -1534,7 +1536,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>CIDET · IA en local · Classe 1</t>
         </is>
@@ -1552,7 +1554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F30"/>
+  <dimension ref="B2:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1561,6 +1563,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1571,156 +1574,184 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Quantització</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Bits</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Bytes/paràmetre</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Mida relativa</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>Pèrdua de qualitat orientativa</t>
         </is>
       </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>Contextos</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>FP16</t>
         </is>
       </c>
-      <c r="C5" s="29" t="n">
+      <c r="C5" s="28" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="29" t="inlineStr">
+      <c r="E5" s="28" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Cap (referència)</t>
         </is>
       </c>
+      <c r="H5" s="31" t="n">
+        <v>2048</v>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="28" t="n">
         <v>8</v>
       </c>
       <c r="D6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>50 %</t>
         </is>
       </c>
-      <c r="F6" s="27" t="inlineStr">
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>Pràcticament imperceptible</t>
         </is>
       </c>
+      <c r="H6" s="31" t="n">
+        <v>4096</v>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="28" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="30" t="n">
         <v>0.75</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>38 %</t>
         </is>
       </c>
-      <c r="F7" s="27" t="inlineStr">
+      <c r="F7" s="26" t="inlineStr">
         <is>
           <t>Molt petita</t>
         </is>
       </c>
+      <c r="H7" s="31" t="n">
+        <v>8192</v>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="25" t="inlineStr">
         <is>
           <t>25 %</t>
         </is>
       </c>
-      <c r="F8" s="24" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>Petita — el punt dolç (Q4_K_M)</t>
         </is>
       </c>
+      <c r="H8" s="31" t="n">
+        <v>16384</v>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="28" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="30" t="n">
         <v>0.4</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
         <is>
           <t>20 %</t>
         </is>
       </c>
-      <c r="F9" s="27" t="inlineStr">
+      <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Notable: comença a fallar en raonament</t>
         </is>
       </c>
+      <c r="H9" s="31" t="n">
+        <v>32768</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="H10" s="31" t="n">
+        <v>65536</v>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="33" t="inlineStr">
         <is>
           <t>Q4_K_M és el punt dolç</t>
         </is>
       </c>
+      <c r="H11" s="31" t="n">
+        <v>131072</v>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>Per al 95 % dels casos d'empresa, la resposta és RAG, no fine-tuning.</t>
         </is>
@@ -1732,76 +1763,76 @@
           <t>LES FÓRMULES DEL CURS</t>
         </is>
       </c>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="34" t="n"/>
-      <c r="E14" s="34" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
       <c r="F14" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B16" s="36" t="inlineStr">
         <is>
           <t>VRAM_pesos (GB) ≈ paràmetres (B) × bytes/paràmetre × 1,1</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="35" t="inlineStr">
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>tokens/s ≈ amplada de banda (GB/s) ÷ mida del model (GB)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="35" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
         <is>
           <t>VRAM_context (GB) ≈ 0,1–0,2 GB per cada 1.000 tokens  (la meitat amb KV cache Q8)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>Regles pràctiques</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="37" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>· El 1,1 de la fórmula és el sobrecost real: activacions, buffers i fragmentació.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="37" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>· Per a assistents d'empresa, temperatura 0–0,3.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="37" t="inlineStr">
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>· El català tokenitza pitjor que l'anglès: més context consumit i, per tant, més lent.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="37" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>· El rendiment real queda entre el 60 % i el 80 % del teòric.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="37" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>· Les Blackwell accelen FP8/FP4 per maquinari; Ampere no.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>CIDET · IA en local · Classe 1</t>
         </is>
@@ -1862,289 +1893,289 @@
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Par. (B)</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Quant.</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="F5" s="23" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>VRAM pesos</t>
         </is>
       </c>
-      <c r="G5" s="23" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>VRAM ctx</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>VRAM teòrica</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>VRAM real (Ollama)</t>
         </is>
       </c>
-      <c r="J5" s="23" t="inlineStr">
+      <c r="J5" s="22" t="inlineStr">
         <is>
           <t>RTX 3060 12GB</t>
         </is>
       </c>
-      <c r="K5" s="23" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>RTX 5070 12GB</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="L5" s="22" t="inlineStr">
         <is>
           <t>RTX 5060 Ti 16GB</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Qwen3 14B</t>
         </is>
       </c>
-      <c r="C6" s="38" t="n">
+      <c r="C6" s="39" t="n">
         <v>14</v>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="27" t="n">
         <v>8192</v>
       </c>
-      <c r="F6" s="39">
+      <c r="F6" s="40">
         <f>C6*VLOOKUP(D6,Referencia!$B$5:$D$9,3,FALSE)*1.1</f>
         <v/>
       </c>
-      <c r="G6" s="39">
+      <c r="G6" s="40">
         <f>E6/1000*0.15*1</f>
         <v/>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="40">
         <f>F6+G6</f>
         <v/>
       </c>
-      <c r="I6" s="40" t="n">
+      <c r="I6" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="J6" s="29">
+      <c r="J6" s="28">
         <f>IF(12-$I6&lt;0,"✘ No",IF(12-$I6&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="K6" s="29">
+      <c r="K6" s="28">
         <f>IF(12-$I6&lt;0,"✘ No",IF(12-$I6&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="L6" s="29">
+      <c r="L6" s="28">
         <f>IF(16-$I6&lt;0,"✘ No",IF(16-$I6&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Gemma 4 26B-A4B</t>
         </is>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="39" t="n">
         <v>26</v>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="28" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="27" t="n">
         <v>8192</v>
       </c>
-      <c r="F7" s="39">
+      <c r="F7" s="40">
         <f>C7*VLOOKUP(D7,Referencia!$B$5:$D$9,3,FALSE)*1.1</f>
         <v/>
       </c>
-      <c r="G7" s="39">
+      <c r="G7" s="40">
         <f>E7/1000*0.15*1</f>
         <v/>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="40">
         <f>F7+G7</f>
         <v/>
       </c>
-      <c r="I7" s="40" t="n">
+      <c r="I7" s="41" t="n">
         <v>15.5</v>
       </c>
-      <c r="J7" s="29">
+      <c r="J7" s="28">
         <f>IF(12-$I7&lt;0,"✘ No",IF(12-$I7&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="K7" s="29">
+      <c r="K7" s="28">
         <f>IF(12-$I7&lt;0,"✘ No",IF(12-$I7&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="L7" s="29">
+      <c r="L7" s="28">
         <f>IF(16-$I7&lt;0,"✘ No",IF(16-$I7&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Qwen3.6 27B</t>
         </is>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C8" s="39" t="n">
         <v>27</v>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="28" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="27" t="n">
         <v>8192</v>
       </c>
-      <c r="F8" s="39">
+      <c r="F8" s="40">
         <f>C8*VLOOKUP(D8,Referencia!$B$5:$D$9,3,FALSE)*1.1</f>
         <v/>
       </c>
-      <c r="G8" s="39">
+      <c r="G8" s="40">
         <f>E8/1000*0.15*1</f>
         <v/>
       </c>
-      <c r="H8" s="39">
+      <c r="H8" s="40">
         <f>F8+G8</f>
         <v/>
       </c>
-      <c r="I8" s="40" t="n">
+      <c r="I8" s="41" t="n">
         <v>18.2</v>
       </c>
-      <c r="J8" s="29">
+      <c r="J8" s="28">
         <f>IF(12-$I8&lt;0,"✘ No",IF(12-$I8&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="K8" s="29">
+      <c r="K8" s="28">
         <f>IF(12-$I8&lt;0,"✘ No",IF(12-$I8&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
-      <c r="L8" s="29">
+      <c r="L8" s="28">
         <f>IF(16-$I8&lt;0,"✘ No",IF(16-$I8&gt;1.5,"✔ Sí","⚠ Just"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="41" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t>Com es llegeix això</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>· Qwen3 14B Q4 amb 8k de context: la fórmula dóna ~8,9 GB, però mesurat a Ollama en surten ~11 GB.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="37" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">   Just a la 5070 (12 GB): arrenca, però sense marge. Còmode a la 5060 Ti (16 GB).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="37" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>· Gemma 4 26B-A4B Q4 → ~15,5 GB. Només a la 5060 Ti, i molt just.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="37" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>· Qwen3.6 27B Q4 → ~18 GB. A cap de les tres GPU de l'aula.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="37" t="inlineStr"/>
+      <c r="B15" s="38" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="41" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>Per què la teòrica i la real no coincideixen?</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>· Q4_K_M no són 0,5 bytes/paràmetre exactes: barreja blocs de 4, 5 i 6 bits i surt a ~0,6 de mitjana.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="37" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>· El runtime (Ollama/llama.cpp) reserva els seus propis búfers de càlcul, a banda de pesos i KV cache.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="37" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>· La fórmula del curs és per DIMENSIONAR de pressa, no per predir al decigram.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="37" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">   Regla de butxaca: si el marge teòric és &lt; 2 GB, considera-ho «just» i mesura-ho abans de prometre res.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="37" t="inlineStr"/>
+      <c r="B21" s="38" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="B22" s="41" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t>Conclusió del curs: amb 12–16 GB, la franja útil és 7B–14B en Q4.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="37" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>Per a més, o compres més VRAM, o acceptes offload a CPU i la lentitud que comporta.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>CIDET · IA en local · Classe 1</t>
         </is>

</xml_diff>